<commit_message>
add ignore empty lines in excel file
</commit_message>
<xml_diff>
--- a/src/test/resources/customers-1000.xlsx
+++ b/src/test/resources/customers-1000.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/songzou/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/songzou/Documents/IdeaProjects/compressed-table/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C093B4F-09E3-3543-85B7-9FA5BAD9BC8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA70BF01-8D9D-934D-B732-F5BA908C9252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="960" windowWidth="25040" windowHeight="14500"/>
+    <workbookView xWindow="480" yWindow="960" windowWidth="25040" windowHeight="14500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="customers-1000" sheetId="1" r:id="rId1"/>
@@ -24218,7 +24218,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -24759,9 +24759,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -24799,7 +24799,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -24905,7 +24905,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -25047,14 +25047,14 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L1001"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -25590,7 +25590,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>

</xml_diff>